<commit_message>
update mongodb connection to speed up
</commit_message>
<xml_diff>
--- a/output/model_results/asset_inputs_summary.xlsx
+++ b/output/model_results/asset_inputs_summary.xlsx
@@ -636,8 +636,10 @@
       <c r="I2" t="n">
         <v>95</v>
       </c>
-      <c r="J2" t="n">
-        <v>1.6</v>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -910,7 +912,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>{'total_capex': 500.0, 'debt_amount': 333.8874816894532, 'equity_amount': 166.11251831054688, 'gearing': 0.6677749633789064}</t>
+          <t>{'total_capex': 500, 'debt_amount': 333.8874816894532, 'equity_amount': 166.11251831054688, 'gearing': 0.6677749633789064}</t>
         </is>
       </c>
       <c r="W4" t="n">
@@ -1721,13 +1723,13 @@
         <v>238.6</v>
       </c>
       <c r="C2" t="n">
-        <v>137.8312205505371</v>
+        <v>155.0894083786011</v>
       </c>
       <c r="D2" t="n">
-        <v>100.7687794494629</v>
+        <v>83.51059162139892</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5776664733886719</v>
+        <v>0.6499975204467774</v>
       </c>
     </row>
     <row r="3">
@@ -1886,7 +1888,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.1088771493647892</v>
+        <v>0.1120658344049389</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update calculations, asset defaults, and add IRR diagnostic tools
</commit_message>
<xml_diff>
--- a/output/model_results/asset_inputs_summary.xlsx
+++ b/output/model_results/asset_inputs_summary.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV2"/>
+  <dimension ref="A1:AQ9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -520,157 +520,132 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
+          <t>contracts</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>lastUpdated</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>costAssumptions</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>assetStartDate</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
           <t>durationHours</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>contracts</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>capex</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>operatingCosts</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>operatingCostEscalation</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>terminalValue</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>maxGearing</t>
-        </is>
-      </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>targetDSCRContract</t>
+          <t>cost_operatingCosts</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>targetDSCRMerchant</t>
+          <t>cost_operatingCostEscalation</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>interestRate</t>
+          <t>cost_terminalValue</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>tenorYears</t>
+          <t>cost_capex</t>
         </is>
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
-          <t>debtStructure</t>
+          <t>cost_maxGearing</t>
         </is>
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>cost_targetDSCRContract</t>
         </is>
       </c>
       <c r="AE1" s="1" t="inlineStr">
         <is>
-          <t>lastUpdated</t>
+          <t>cost_targetDSCRMerchant</t>
         </is>
       </c>
       <c r="AF1" s="1" t="inlineStr">
         <is>
-          <t>costAssumptions</t>
+          <t>cost_interestRate</t>
         </is>
       </c>
       <c r="AG1" s="1" t="inlineStr">
         <is>
-          <t>cost_capex</t>
+          <t>cost_tenorYears</t>
         </is>
       </c>
       <c r="AH1" s="1" t="inlineStr">
         <is>
-          <t>cost_operatingCosts</t>
+          <t>cost_calculatedGearing</t>
         </is>
       </c>
       <c r="AI1" s="1" t="inlineStr">
         <is>
-          <t>cost_operatingCostEscalation</t>
+          <t>cost_debtStructure</t>
         </is>
       </c>
       <c r="AJ1" s="1" t="inlineStr">
         <is>
-          <t>cost_terminalValue</t>
+          <t>debt_total_capex</t>
         </is>
       </c>
       <c r="AK1" s="1" t="inlineStr">
         <is>
-          <t>cost_maxGearing</t>
+          <t>debt_debt_amount</t>
         </is>
       </c>
       <c r="AL1" s="1" t="inlineStr">
         <is>
-          <t>cost_targetDSCRContract</t>
+          <t>debt_equity_amount</t>
         </is>
       </c>
       <c r="AM1" s="1" t="inlineStr">
         <is>
-          <t>cost_targetDSCRMerchant</t>
+          <t>debt_gearing</t>
         </is>
       </c>
       <c r="AN1" s="1" t="inlineStr">
         <is>
-          <t>cost_interestRate</t>
+          <t>asset_equity_irr</t>
         </is>
       </c>
       <c r="AO1" s="1" t="inlineStr">
         <is>
-          <t>cost_tenorYears</t>
+          <t>portfolio</t>
         </is>
       </c>
       <c r="AP1" s="1" t="inlineStr">
         <is>
-          <t>cost_debtStructure</t>
+          <t>capacityFactor</t>
         </is>
       </c>
       <c r="AQ1" s="1" t="inlineStr">
         <is>
-          <t>debt_total_capex</t>
-        </is>
-      </c>
-      <c r="AR1" s="1" t="inlineStr">
-        <is>
-          <t>debt_debt_amount</t>
-        </is>
-      </c>
-      <c r="AS1" s="1" t="inlineStr">
-        <is>
-          <t>debt_equity_amount</t>
-        </is>
-      </c>
-      <c r="AT1" s="1" t="inlineStr">
-        <is>
-          <t>debt_gearing</t>
-        </is>
-      </c>
-      <c r="AU1" s="1" t="inlineStr">
-        <is>
-          <t>asset_equity_irr</t>
-        </is>
-      </c>
-      <c r="AV1" s="1" t="inlineStr">
-        <is>
-          <t>portfolio</t>
+          <t>debtSizingResults</t>
         </is>
       </c>
     </row>
@@ -680,27 +655,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>Templers BESS</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>Templers BESS</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>SA</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>solar</t>
+          <t>storage</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>111</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -709,144 +684,1172 @@
       <c r="H2" t="n">
         <v>95</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2024-03-01</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>17</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2025-08-01</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>293</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>[{'id': '1', 'counterparty': 'ZEN Tolling', 'type': 'tolling', 'buyersPercentage': 100, 'strikePrice': '23', 'indexation': 2.5, 'indexationReferenceYear': 2025, 'startDate': '2025-08-01', 'endDate': '2035-07-31', 'hasFloor': False, 'floorValue': '0', 'EnergyPrice': '', 'greenPrice': ''}]</t>
+        </is>
+      </c>
+      <c r="S2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>2025-07-14T11:34:55.837Z</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>{'operatingCosts': 4.06, 'operatingCostEscalation': 2.5, 'terminalValue': 51, 'capex': 238.6, 'maxGearing': 0.65, 'targetDSCRContract': 1.4, 'targetDSCRMerchant': 1.8, 'interestRate': 0.06, 'tenorYears': 20, 'calculatedGearing': 0.65, 'debtStructure': 'sculpting'}</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>2025-08-01</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>2.64</t>
+        </is>
+      </c>
+      <c r="Y2" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>51</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>238.6</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>20</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>sculpting</t>
+        </is>
+      </c>
+      <c r="AJ2" t="n">
+        <v>238.6</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>155.0894083786011</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>83.51059162139892</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>0.6499975204467774</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>0.1436087041880745</v>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>ZEBRE</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Solar River Solar</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Solar River Solar</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>solar</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>232</v>
+      </c>
+      <c r="G3" t="n">
+        <v>30</v>
+      </c>
+      <c r="H3" t="n">
+        <v>97</v>
+      </c>
+      <c r="I3" t="n">
         <v>0.5</v>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>2025-01-01</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2025-10-01</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>21</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2027-07-01</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>[{'id': '1', 'counterparty': None, 'type': 'bundled', 'buyersPercentage': 100, 'shape': 'flat', 'strikePrice': 50, 'greenPrice': 5, 'EnergyPrice': 45, 'indexation': '2.5', 'indexationReferenceYear': '2025', 'settlementFormula': '', 'hasFloor': False, 'floorValue': '', 'startDate': '2027-07-01', 'endDate': '2037-06-30'}]</t>
+        </is>
+      </c>
+      <c r="S3" t="n">
+        <v>2</v>
+      </c>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>{'operatingCosts': 3.25, 'operatingCostEscalation': 2.5, 'terminalValue': 0, 'capex': 208.3, 'maxGearing': 0.7, 'targetDSCRContract': 1.4, 'targetDSCRMerchant': 1.8, 'interestRate': 0.06, 'tenorYears': 22, 'calculatedGearing': 0.7, 'debtStructure': 'sculpting'}</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>2027-07-01</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>208.3</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>22</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>sculpting</t>
+        </is>
+      </c>
+      <c r="AJ3" t="n">
+        <v>208.3</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>145.8094437789917</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>62.49055622100832</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>0.699997329711914</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>0.2838806754680757</v>
+      </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>ZEBRE</t>
+        </is>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>{'total_capex': 208.3, 'debt_amount': 145.8094437789917, 'equity_amount': 62.49055622100832, 'gearing': 0.699997329711914}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Solar River BESS</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Solar River BESS</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>256</v>
+      </c>
+      <c r="G4" t="n">
+        <v>25</v>
+      </c>
+      <c r="H4" t="n">
+        <v>97</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2025-10-01</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>21</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2027-07-01</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="n">
+        <v>656</v>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>[{'id': '1', 'counterparty': 'ZEN Tolling', 'type': 'tolling', 'buyersPercentage': 100, 'shape': 'flat', 'strikePrice': 24, 'greenPrice': None, 'EnergyPrice': None, 'indexation': 2.5, 'indexationReferenceYear': '2025', 'settlementFormula': '', 'hasFloor': False, 'floorValue': '', 'startDate': '2027-07-01', 'endDate': '2037-06-30'}]</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>3</v>
+      </c>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>{'operatingCosts': 10.01, 'operatingCostEscalation': 2.5, 'terminalValue': 119, 'capex': 500, 'maxGearing': 0.7, 'targetDSCRContract': 1.4, 'targetDSCRMerchant': 1.8, 'interestRate': 0.06, 'tenorYears': 20, 'calculatedGearing': 0.7, 'debtStructure': 'sculpting'}</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>2027-07-01</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>2.56</t>
+        </is>
+      </c>
+      <c r="Y4" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>119</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>500</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>20</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>sculpting</t>
+        </is>
+      </c>
+      <c r="AJ4" t="n">
+        <v>500</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>337.9670143127441</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>162.0329856872559</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>0.6759340286254882</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>0.1623527630417089</v>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>ZEBRE</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>{'total_capex': 500, 'debt_amount': 333.8874816894532, 'equity_amount': 166.11251831054688, 'gearing': 0.6677749633789064}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Wagga North</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Wagga North</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>NSW</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>105</v>
+      </c>
+      <c r="G5" t="n">
+        <v>25</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>21</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2028-08-01</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="n">
+        <v>420</v>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>[{'id': '1', 'counterparty': 'ZEN', 'type': 'tolling', 'buyersPercentage': 100, 'shape': 'flat', 'strikePrice': 20, 'greenPrice': '', 'EnergyPrice': '', 'indexation': 2.5, 'indexationReferenceYear': '2025', 'settlementFormula': '', 'hasFloor': False, 'floorValue': '', 'startDate': '2028-08-01', 'endDate': '2038-07-31'}]</t>
+        </is>
+      </c>
+      <c r="S5" t="n">
+        <v>4</v>
+      </c>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>{'operatingCosts': 3.23, 'operatingCostEscalation': 2.5, 'terminalValue': 49, 'capex': 246.8, 'maxGearing': 0.65, 'targetDSCRContract': 1.4, 'targetDSCRMerchant': 1.8, 'interestRate': 0.06, 'tenorYears': 20, 'calculatedGearing': 0.65, 'debtStructure': 'sculpting'}</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>NSW</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>2028-08-01</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>4.00</t>
+        </is>
+      </c>
+      <c r="Y5" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>49</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>246.8</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>20</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>sculpting</t>
+        </is>
+      </c>
+      <c r="AJ5" t="n">
+        <v>246.8</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>160.4193880462647</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>86.38061195373534</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>0.6499975204467774</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>0.1305817350477535</v>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>ZEBRE</t>
+        </is>
+      </c>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>{'total_capex': 246.8, 'debt_amount': 159.657505645752, 'equity_amount': 87.14249435424802, 'gearing': 0.6469104766845705}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Noblevale</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Noblevale</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>QLD</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>180</v>
+      </c>
+      <c r="G6" t="n">
+        <v>25</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>21</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2028-05-01</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="n">
+        <v>360</v>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>[{'id': '1', 'counterparty': 'ZEN', 'type': 'tolling', 'buyersPercentage': 100, 'shape': 'flat', 'strikePrice': 18, 'greenPrice': '', 'EnergyPrice': '', 'indexation': 2.5, 'indexationReferenceYear': '2025', 'settlementFormula': '', 'hasFloor': False, 'floorValue': '', 'startDate': '2028-05-01', 'endDate': '2038-04-30'}]</t>
+        </is>
+      </c>
+      <c r="S6" t="n">
+        <v>5</v>
+      </c>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>{'operatingCosts': 5.19, 'operatingCostEscalation': 2.5, 'terminalValue': 83, 'capex': 296.6, 'maxGearing': 0.65, 'targetDSCRContract': 1.4, 'targetDSCRMerchant': 1.8, 'interestRate': 0.06, 'tenorYears': 20, 'calculatedGearing': 0.65, 'debtStructure': 'sculpting'}</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>QLD</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>2028-05-01</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="Y6" t="n">
+        <v>5.19</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>83</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>296.6</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>20</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>sculpting</t>
+        </is>
+      </c>
+      <c r="AJ6" t="n">
+        <v>296.6</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>192.7892645645142</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>103.8107354354859</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>0.6499975204467774</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>0.1607519897242499</v>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>ZEBRE</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>{'total_capex': 296.6, 'debt_amount': 192.78926456451418, 'equity_amount': 103.81073543548585, 'gearing': 0.6499975204467774}</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Hookey Creek (BESS)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Hookey Creek (BESS)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>NSW</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>200</v>
+      </c>
+      <c r="G7" t="n">
+        <v>25</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>24</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2028-05-01</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="n">
+        <v>800</v>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>[{'id': '1', 'counterparty': 'ZEN', 'type': 'tolling', 'buyersPercentage': 100, 'shape': 'flat', 'strikePrice': 20, 'greenPrice': '', 'EnergyPrice': '', 'indexation': 2.5, 'indexationReferenceYear': '2025', 'settlementFormula': '', 'hasFloor': False, 'floorValue': '', 'startDate': '2028-05-01', 'endDate': '2038-04-30'}]</t>
+        </is>
+      </c>
+      <c r="S7" t="n">
+        <v>6</v>
+      </c>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>{'operatingCosts': 5.95, 'operatingCostEscalation': 2.5, 'terminalValue': 93, 'capex': 452.7, 'maxGearing': 0.65, 'targetDSCRContract': 1.4, 'targetDSCRMerchant': 1.8, 'interestRate': 0.06, 'tenorYears': 20, 'calculatedGearing': 0.65, 'debtStructure': 'sculpting'}</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>NSW</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>2028-05-01</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>4.00</t>
+        </is>
+      </c>
+      <c r="Y7" t="n">
+        <v>5.95</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>93</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>452.7</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>20</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>sculpting</t>
+        </is>
+      </c>
+      <c r="AJ7" t="n">
+        <v>452.7</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>294.2544387531281</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>158.445561246872</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>0.6499987602233886</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>0.136922849696032</v>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>ZEBRE</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>{'total_capex': 452.70000000000005, 'debt_amount': 294.25443875312806, 'equity_amount': 158.44556124687196, 'gearing': 0.6499987602233886}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>North Yarragon</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>North Yarragon</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>VIC</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>210</v>
+      </c>
+      <c r="G8" t="n">
+        <v>25</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2027-08-01</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>21</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2029-05-01</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="n">
+        <v>840</v>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>[{'id': '1', 'counterparty': 'ZEN Tolling', 'type': 'tolling', 'buyersPercentage': 100, 'shape': 'flat', 'strikePrice': 20, 'greenPrice': '', 'EnergyPrice': '', 'indexation': 2.5, 'indexationReferenceYear': '2025', 'settlementFormula': '', 'hasFloor': False, 'floorValue': '', 'startDate': '2029-05-01', 'endDate': '2039-04-30'}]</t>
+        </is>
+      </c>
+      <c r="S8" t="n">
+        <v>7</v>
+      </c>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>{'operatingCosts': 6.05, 'operatingCostEscalation': 2.5, 'terminalValue': 97, 'capex': 512.7, 'maxGearing': 0.65, 'targetDSCRContract': 1.4, 'targetDSCRMerchant': 1.8, 'interestRate': 0.06, 'tenorYears': 20, 'calculatedGearing': 0.65, 'debtStructure': 'sculpting'}</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>VIC</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>2029-05-01</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>4.00</t>
+        </is>
+      </c>
+      <c r="Y8" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>97</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>512.7</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>20</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>sculpting</t>
+        </is>
+      </c>
+      <c r="AJ8" t="n">
+        <v>512.7000000000002</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>333.2543643665313</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>179.4456356334688</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>0.6499987602233883</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>0.1324552854535143</v>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>ZEBRE</t>
+        </is>
+      </c>
+      <c r="AP8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>{'total_capex': 512.7000000000002, 'debt_amount': 333.2543643665313, 'equity_amount': 179.44563563346878, 'gearing': 0.6499987602233883}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Yarraville</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Yarraville</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>VIC</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G9" t="n">
+        <v>25</v>
+      </c>
+      <c r="H9" t="n">
+        <v>97.5</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>12</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2028-01-01</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="n">
+        <v>210</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>[{'id': '1', 'counterparty': 'ZEN Tolling', 'type': 'tolling', 'buyersPercentage': 100, 'shape': 'flat', 'strikePrice': 21, 'greenPrice': '', 'EnergyPrice': '', 'indexation': '2.5', 'indexationReferenceYear': '2025', 'settlementFormula': '', 'hasFloor': False, 'floorValue': '', 'startDate': '2028-01-01', 'endDate': '2037-12-31'}]</t>
+        </is>
+      </c>
+      <c r="S9" t="n">
+        <v>8</v>
+      </c>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>{'capex': 141.5, 'operatingCosts': 2.2, 'operatingCostEscalation': 2.5, 'terminalValue': 32, 'maxGearing': 0.7, 'targetDSCRContract': 1.4, 'targetDSCRMerchant': 2, 'interestRate': 0.06, 'tenorYears': 18, 'debtStructure': 'sculpting', 'calculatedGearing': 0.7}</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>VIC</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>2028-01-01</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="Y9" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>32</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>141.5</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AG9" t="n">
         <v>18</v>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="T2" t="n">
-        <v>134.4</v>
-      </c>
-      <c r="U2" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="V2" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="W2" t="n">
-        <v>0</v>
-      </c>
-      <c r="X2" t="n">
+      <c r="AH9" t="n">
         <v>0.7</v>
       </c>
-      <c r="Y2" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>20</v>
-      </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AI9" t="inlineStr">
         <is>
           <t>sculpting</t>
         </is>
       </c>
-      <c r="AD2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>2025-12-03T23:17:05.821Z</t>
-        </is>
-      </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>{'capex': 1.3, 'operatingCosts': 0.06, 'operatingCostEscalation': 2.5, 'terminalValue': 0, 'maxGearing': 0.7, 'targetDSCRContract': 1.4, 'targetDSCRMerchant': 1.8, 'interestRate': 0.06, 'tenorYears': 20, 'debtStructure': 'sculpting'}</t>
-        </is>
-      </c>
-      <c r="AG2" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="AH2" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="AI2" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="AJ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK2" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AL2" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="AM2" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="AN2" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="AO2" t="n">
-        <v>20</v>
-      </c>
-      <c r="AP2" t="inlineStr">
-        <is>
-          <t>sculpting</t>
-        </is>
-      </c>
-      <c r="AQ2" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="AR2" t="n">
-        <v>0.9091113281249998</v>
-      </c>
-      <c r="AS2" t="n">
-        <v>0.3908886718750003</v>
-      </c>
-      <c r="AT2" t="n">
-        <v>0.6993164062499997</v>
-      </c>
-      <c r="AU2" t="n">
-        <v>1.142685093689932</v>
-      </c>
-      <c r="AV2" t="inlineStr">
-        <is>
-          <t>Test2</t>
+      <c r="AJ9" t="n">
+        <v>141.5</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>95.60102386474611</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>45.89897613525388</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>0.6756256103515627</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>0.1721991906314946</v>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>ZEBRE</t>
+        </is>
+      </c>
+      <c r="AP9" t="inlineStr"/>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t>{'total_capex': 141.5, 'debt_amount': 94.51887359619141, 'equity_amount': 46.98112640380858, 'gearing': 0.6679779052734376}</t>
         </is>
       </c>
     </row>
@@ -1019,7 +2022,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1052,20 +2055,153 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>Templers BESS</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.3</v>
+        <v>238.6</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9091113281249998</v>
+        <v>155.0894083786011</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3908886718750003</v>
+        <v>83.51059162139892</v>
       </c>
       <c r="E2" t="n">
-        <v>0.6993164062499997</v>
+        <v>0.6499975204467774</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Solar River Solar</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>208.3</v>
+      </c>
+      <c r="C3" t="n">
+        <v>145.8094437789917</v>
+      </c>
+      <c r="D3" t="n">
+        <v>62.49055622100832</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.699997329711914</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Solar River BESS</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>500</v>
+      </c>
+      <c r="C4" t="n">
+        <v>337.9670143127441</v>
+      </c>
+      <c r="D4" t="n">
+        <v>162.0329856872559</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.6759340286254882</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Wagga North</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>246.8</v>
+      </c>
+      <c r="C5" t="n">
+        <v>160.4193880462647</v>
+      </c>
+      <c r="D5" t="n">
+        <v>86.38061195373534</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.6499975204467774</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Noblevale</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>296.6</v>
+      </c>
+      <c r="C6" t="n">
+        <v>192.7892645645142</v>
+      </c>
+      <c r="D6" t="n">
+        <v>103.8107354354859</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.6499975204467774</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Hookey Creek (BESS)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>452.7</v>
+      </c>
+      <c r="C7" t="n">
+        <v>294.2544387531281</v>
+      </c>
+      <c r="D7" t="n">
+        <v>158.445561246872</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.6499987602233886</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>North Yarragon</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>512.7000000000002</v>
+      </c>
+      <c r="C8" t="n">
+        <v>333.2543643665313</v>
+      </c>
+      <c r="D8" t="n">
+        <v>179.4456356334688</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.6499987602233883</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Yarraville</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>141.5</v>
+      </c>
+      <c r="C9" t="n">
+        <v>95.60102386474611</v>
+      </c>
+      <c r="D9" t="n">
+        <v>45.89897613525388</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.6756256103515627</v>
       </c>
     </row>
   </sheetData>
@@ -1091,7 +2227,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1.142685093689932</v>
+        <v>0.158395181268125</v>
       </c>
     </row>
   </sheetData>
@@ -1105,7 +2241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1125,7 +2261,63 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>1.142685093689932</v>
+        <v>0.1436087041880745</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.2838806754680757</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.1623527630417089</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.1305817350477535</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0.1607519897242499</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.136922849696032</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.1324552854535143</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.1721991906314946</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Run backend and frontend servers, update backend imports and start scripts
</commit_message>
<xml_diff>
--- a/output/model_results/asset_inputs_summary.xlsx
+++ b/output/model_results/asset_inputs_summary.xlsx
@@ -520,132 +520,132 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
+          <t>durationHours</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
           <t>contracts</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>lastUpdated</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>costAssumptions</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>cost_operatingCosts</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>cost_operatingCostEscalation</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>cost_terminalValue</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>cost_capex</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>cost_maxGearing</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>cost_targetDSCRContract</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>cost_targetDSCRMerchant</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>cost_interestRate</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>cost_tenorYears</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>cost_calculatedGearing</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>cost_debtStructure</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>debt_total_capex</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>debt_debt_amount</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>debt_equity_amount</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>debt_gearing</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>asset_equity_irr</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>portfolio</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>capacityFactor</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>debtSizingResults</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>state</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>assetStartDate</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>durationHours</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>cost_operatingCosts</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>cost_operatingCostEscalation</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>cost_terminalValue</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>cost_capex</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>cost_maxGearing</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>cost_targetDSCRContract</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>cost_targetDSCRMerchant</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>cost_interestRate</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>cost_tenorYears</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>cost_calculatedGearing</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>cost_debtStructure</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>debt_total_capex</t>
-        </is>
-      </c>
-      <c r="AK1" s="1" t="inlineStr">
-        <is>
-          <t>debt_debt_amount</t>
-        </is>
-      </c>
-      <c r="AL1" s="1" t="inlineStr">
-        <is>
-          <t>debt_equity_amount</t>
-        </is>
-      </c>
-      <c r="AM1" s="1" t="inlineStr">
-        <is>
-          <t>debt_gearing</t>
-        </is>
-      </c>
-      <c r="AN1" s="1" t="inlineStr">
-        <is>
-          <t>asset_equity_irr</t>
-        </is>
-      </c>
-      <c r="AO1" s="1" t="inlineStr">
-        <is>
-          <t>portfolio</t>
-        </is>
-      </c>
-      <c r="AP1" s="1" t="inlineStr">
-        <is>
-          <t>capacityFactor</t>
-        </is>
-      </c>
-      <c r="AQ1" s="1" t="inlineStr">
-        <is>
-          <t>debtSizingResults</t>
         </is>
       </c>
     </row>
@@ -713,92 +713,84 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>[{'id': '1', 'counterparty': 'ZEN Tolling', 'type': 'tolling', 'buyersPercentage': 100, 'strikePrice': '23', 'indexation': 2.5, 'indexationReferenceYear': 2025, 'startDate': '2025-08-01', 'endDate': '2035-07-31', 'hasFloor': False, 'floorValue': '0', 'EnergyPrice': '', 'greenPrice': ''}]</t>
-        </is>
-      </c>
-      <c r="S2" t="n">
+          <t>2.64</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>[{'id': '1', 'counterparty': 'ZEN Tolling', 'type': 'tolling', 'buyersPercentage': 100, 'strikePrice': '23.5', 'indexation': 2.5, 'indexationReferenceYear': 2025, 'startDate': '2025-12-01', 'endDate': '2035-07-31', 'hasFloor': False, 'floorValue': '0', 'EnergyPrice': '', 'greenPrice': ''}]</t>
+        </is>
+      </c>
+      <c r="T2" t="n">
         <v>1</v>
       </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>2025-07-14T11:34:55.837Z</t>
-        </is>
-      </c>
       <c r="U2" t="inlineStr">
         <is>
+          <t>2025-12-04T04:16:53.384Z</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
           <t>{'operatingCosts': 4.06, 'operatingCostEscalation': 2.5, 'terminalValue': 51, 'capex': 238.6, 'maxGearing': 0.65, 'targetDSCRContract': 1.4, 'targetDSCRMerchant': 1.8, 'interestRate': 0.06, 'tenorYears': 20, 'calculatedGearing': 0.65, 'debtStructure': 'sculpting'}</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>SA</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>2025-08-01</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>2.64</t>
-        </is>
+      <c r="W2" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="X2" t="n">
+        <v>2.5</v>
       </c>
       <c r="Y2" t="n">
-        <v>4.06</v>
+        <v>51</v>
       </c>
       <c r="Z2" t="n">
-        <v>2.5</v>
+        <v>238.6</v>
       </c>
       <c r="AA2" t="n">
-        <v>51</v>
+        <v>0.65</v>
       </c>
       <c r="AB2" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>20</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>sculpting</t>
+        </is>
+      </c>
+      <c r="AH2" t="n">
         <v>238.6</v>
       </c>
-      <c r="AC2" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="AE2" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="AF2" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="AG2" t="n">
-        <v>20</v>
-      </c>
-      <c r="AH2" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>sculpting</t>
-        </is>
+      <c r="AI2" t="n">
+        <v>155.0894083786011</v>
       </c>
       <c r="AJ2" t="n">
-        <v>238.6</v>
+        <v>83.51059162139892</v>
       </c>
       <c r="AK2" t="n">
-        <v>155.0894083786011</v>
+        <v>0.6499975204467774</v>
       </c>
       <c r="AL2" t="n">
-        <v>83.51059162139892</v>
-      </c>
-      <c r="AM2" t="n">
-        <v>0.6499975204467774</v>
-      </c>
-      <c r="AN2" t="n">
-        <v>0.1436087041880745</v>
-      </c>
-      <c r="AO2" t="inlineStr">
+        <v>0.09946314289147172</v>
+      </c>
+      <c r="AM2" t="inlineStr">
         <is>
           <t>ZEBRE</t>
         </is>
       </c>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
       <c r="AP2" t="inlineStr"/>
       <c r="AQ2" t="inlineStr"/>
     </row>
@@ -826,8 +818,10 @@
           <t>solar</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>232</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>232</t>
+        </is>
       </c>
       <c r="G3" t="n">
         <v>30</v>
@@ -872,96 +866,84 @@
         </is>
       </c>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>[{'id': '1', 'counterparty': None, 'type': 'bundled', 'buyersPercentage': 100, 'shape': 'flat', 'strikePrice': 50, 'greenPrice': 5, 'EnergyPrice': 45, 'indexation': '2.5', 'indexationReferenceYear': '2025', 'settlementFormula': '', 'hasFloor': False, 'floorValue': '', 'startDate': '2027-07-01', 'endDate': '2037-06-30'}]</t>
-        </is>
-      </c>
-      <c r="S3" t="n">
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>[{'id': '1', 'counterparty': '', 'type': 'bundled', 'buyersPercentage': 100, 'strikePrice': '50', 'indexation': '2.5', 'indexationReferenceYear': '2025', 'startDate': '2028-07-01', 'endDate': '2038-06-30', 'hasFloor': False, 'floorValue': '', 'EnergyPrice': '45', 'greenPrice': '5'}]</t>
+        </is>
+      </c>
+      <c r="T3" t="n">
         <v>2</v>
       </c>
-      <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr">
         <is>
+          <t>2025-12-04T04:17:33.719Z</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
           <t>{'operatingCosts': 3.25, 'operatingCostEscalation': 2.5, 'terminalValue': 0, 'capex': 208.3, 'maxGearing': 0.7, 'targetDSCRContract': 1.4, 'targetDSCRMerchant': 1.8, 'interestRate': 0.06, 'tenorYears': 22, 'calculatedGearing': 0.7, 'debtStructure': 'sculpting'}</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>SA</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>2027-07-01</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr"/>
+      <c r="W3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="X3" t="n">
+        <v>2.5</v>
+      </c>
       <c r="Y3" t="n">
-        <v>3.25</v>
+        <v>0</v>
       </c>
       <c r="Z3" t="n">
-        <v>2.5</v>
+        <v>208.3</v>
       </c>
       <c r="AA3" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="AB3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>22</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>sculpting</t>
+        </is>
+      </c>
+      <c r="AH3" t="n">
         <v>208.3</v>
       </c>
-      <c r="AC3" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AD3" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="AE3" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="AF3" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="AG3" t="n">
-        <v>22</v>
-      </c>
-      <c r="AH3" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AI3" t="inlineStr">
-        <is>
-          <t>sculpting</t>
-        </is>
+      <c r="AI3" t="n">
+        <v>145.8094437789917</v>
       </c>
       <c r="AJ3" t="n">
-        <v>208.3</v>
+        <v>62.49055622100832</v>
       </c>
       <c r="AK3" t="n">
-        <v>145.8094437789917</v>
+        <v>0.699997329711914</v>
       </c>
       <c r="AL3" t="n">
-        <v>62.49055622100832</v>
-      </c>
-      <c r="AM3" t="n">
-        <v>0.699997329711914</v>
-      </c>
-      <c r="AN3" t="n">
-        <v>0.2838806754680757</v>
-      </c>
-      <c r="AO3" t="inlineStr">
+        <v>0.2104294561684678</v>
+      </c>
+      <c r="AM3" t="inlineStr">
         <is>
           <t>ZEBRE</t>
         </is>
       </c>
-      <c r="AP3" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="AQ3" t="inlineStr">
-        <is>
-          <t>{'total_capex': 208.3, 'debt_amount': 145.8094437789917, 'equity_amount': 62.49055622100832, 'gearing': 0.699997329711914}</t>
-        </is>
-      </c>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -987,8 +969,10 @@
           <t>storage</t>
         </is>
       </c>
-      <c r="F4" t="n">
-        <v>256</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>256</t>
+        </is>
       </c>
       <c r="G4" t="n">
         <v>25</v>
@@ -1016,99 +1000,93 @@
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="n">
-        <v>656</v>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>656</t>
+        </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>[{'id': '1', 'counterparty': 'ZEN Tolling', 'type': 'tolling', 'buyersPercentage': 100, 'shape': 'flat', 'strikePrice': 24, 'greenPrice': None, 'EnergyPrice': None, 'indexation': 2.5, 'indexationReferenceYear': '2025', 'settlementFormula': '', 'hasFloor': False, 'floorValue': '', 'startDate': '2027-07-01', 'endDate': '2037-06-30'}]</t>
-        </is>
-      </c>
-      <c r="S4" t="n">
+          <t>2.56</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>[{'id': '1', 'counterparty': 'ZEN Tolling', 'type': 'tolling', 'buyersPercentage': 100, 'strikePrice': '21', 'indexation': 2.5, 'indexationReferenceYear': '2025', 'startDate': '2028-07-01', 'endDate': '2038-06-30', 'hasFloor': False, 'floorValue': '', 'EnergyPrice': '', 'greenPrice': ''}]</t>
+        </is>
+      </c>
+      <c r="T4" t="n">
         <v>3</v>
       </c>
-      <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr">
         <is>
+          <t>2025-12-04T04:17:59.013Z</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
           <t>{'operatingCosts': 10.01, 'operatingCostEscalation': 2.5, 'terminalValue': 119, 'capex': 500, 'maxGearing': 0.7, 'targetDSCRContract': 1.4, 'targetDSCRMerchant': 1.8, 'interestRate': 0.06, 'tenorYears': 20, 'calculatedGearing': 0.7, 'debtStructure': 'sculpting'}</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>SA</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>2027-07-01</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>2.56</t>
-        </is>
+      <c r="W4" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="X4" t="n">
+        <v>2.5</v>
       </c>
       <c r="Y4" t="n">
-        <v>10.01</v>
+        <v>119</v>
       </c>
       <c r="Z4" t="n">
-        <v>2.5</v>
+        <v>500</v>
       </c>
       <c r="AA4" t="n">
-        <v>119</v>
+        <v>0.7</v>
       </c>
       <c r="AB4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>20</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>sculpting</t>
+        </is>
+      </c>
+      <c r="AH4" t="n">
         <v>500</v>
       </c>
-      <c r="AC4" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="AE4" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="AF4" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="AG4" t="n">
-        <v>20</v>
-      </c>
-      <c r="AH4" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AI4" t="inlineStr">
-        <is>
-          <t>sculpting</t>
-        </is>
+      <c r="AI4" t="n">
+        <v>297.6076126098633</v>
       </c>
       <c r="AJ4" t="n">
-        <v>500</v>
+        <v>202.3923873901367</v>
       </c>
       <c r="AK4" t="n">
-        <v>337.9670143127441</v>
+        <v>0.5952152252197267</v>
       </c>
       <c r="AL4" t="n">
-        <v>162.0329856872559</v>
-      </c>
-      <c r="AM4" t="n">
-        <v>0.6759340286254882</v>
-      </c>
-      <c r="AN4" t="n">
-        <v>0.1623527630417089</v>
-      </c>
-      <c r="AO4" t="inlineStr">
+        <v>0.07631405246890151</v>
+      </c>
+      <c r="AM4" t="inlineStr">
         <is>
           <t>ZEBRE</t>
         </is>
       </c>
+      <c r="AN4" t="inlineStr"/>
+      <c r="AO4" t="inlineStr"/>
       <c r="AP4" t="inlineStr"/>
-      <c r="AQ4" t="inlineStr">
-        <is>
-          <t>{'total_capex': 500, 'debt_amount': 333.8874816894532, 'equity_amount': 166.11251831054688, 'gearing': 0.6677749633789064}</t>
-        </is>
-      </c>
+      <c r="AQ4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1170,92 +1148,92 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
+          <t>4.00</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
           <t>[{'id': '1', 'counterparty': 'ZEN', 'type': 'tolling', 'buyersPercentage': 100, 'shape': 'flat', 'strikePrice': 20, 'greenPrice': '', 'EnergyPrice': '', 'indexation': 2.5, 'indexationReferenceYear': '2025', 'settlementFormula': '', 'hasFloor': False, 'floorValue': '', 'startDate': '2028-08-01', 'endDate': '2038-07-31'}]</t>
         </is>
       </c>
-      <c r="S5" t="n">
+      <c r="T5" t="n">
         <v>4</v>
       </c>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr">
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr">
         <is>
           <t>{'operatingCosts': 3.23, 'operatingCostEscalation': 2.5, 'terminalValue': 49, 'capex': 246.8, 'maxGearing': 0.65, 'targetDSCRContract': 1.4, 'targetDSCRMerchant': 1.8, 'interestRate': 0.06, 'tenorYears': 20, 'calculatedGearing': 0.65, 'debtStructure': 'sculpting'}</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="W5" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="X5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>49</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>246.8</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>20</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>sculpting</t>
+        </is>
+      </c>
+      <c r="AH5" t="n">
+        <v>246.8</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>121.4581295776367</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>125.3418704223633</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>0.4921318054199219</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>0.08692668341712489</v>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>ZEBRE</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>{'total_capex': 246.8, 'debt_amount': 159.657505645752, 'equity_amount': 87.14249435424802, 'gearing': 0.6469104766845705}</t>
+        </is>
+      </c>
+      <c r="AP5" t="inlineStr">
         <is>
           <t>NSW</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr">
+      <c r="AQ5" t="inlineStr">
         <is>
           <t>2028-08-01</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>4.00</t>
-        </is>
-      </c>
-      <c r="Y5" t="n">
-        <v>3.23</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>49</v>
-      </c>
-      <c r="AB5" t="n">
-        <v>246.8</v>
-      </c>
-      <c r="AC5" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="AD5" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="AE5" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="AF5" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="AG5" t="n">
-        <v>20</v>
-      </c>
-      <c r="AH5" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="AI5" t="inlineStr">
-        <is>
-          <t>sculpting</t>
-        </is>
-      </c>
-      <c r="AJ5" t="n">
-        <v>246.8</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>160.4193880462647</v>
-      </c>
-      <c r="AL5" t="n">
-        <v>86.38061195373534</v>
-      </c>
-      <c r="AM5" t="n">
-        <v>0.6499975204467774</v>
-      </c>
-      <c r="AN5" t="n">
-        <v>0.1305817350477535</v>
-      </c>
-      <c r="AO5" t="inlineStr">
-        <is>
-          <t>ZEBRE</t>
-        </is>
-      </c>
-      <c r="AP5" t="inlineStr"/>
-      <c r="AQ5" t="inlineStr">
-        <is>
-          <t>{'total_capex': 246.8, 'debt_amount': 159.657505645752, 'equity_amount': 87.14249435424802, 'gearing': 0.6469104766845705}</t>
         </is>
       </c>
     </row>
@@ -1319,92 +1297,92 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
           <t>[{'id': '1', 'counterparty': 'ZEN', 'type': 'tolling', 'buyersPercentage': 100, 'shape': 'flat', 'strikePrice': 18, 'greenPrice': '', 'EnergyPrice': '', 'indexation': 2.5, 'indexationReferenceYear': '2025', 'settlementFormula': '', 'hasFloor': False, 'floorValue': '', 'startDate': '2028-05-01', 'endDate': '2038-04-30'}]</t>
         </is>
       </c>
-      <c r="S6" t="n">
+      <c r="T6" t="n">
         <v>5</v>
       </c>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr">
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr">
         <is>
           <t>{'operatingCosts': 5.19, 'operatingCostEscalation': 2.5, 'terminalValue': 83, 'capex': 296.6, 'maxGearing': 0.65, 'targetDSCRContract': 1.4, 'targetDSCRMerchant': 1.8, 'interestRate': 0.06, 'tenorYears': 20, 'calculatedGearing': 0.65, 'debtStructure': 'sculpting'}</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="W6" t="n">
+        <v>5.19</v>
+      </c>
+      <c r="X6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>83</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>296.6</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>20</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>sculpting</t>
+        </is>
+      </c>
+      <c r="AH6" t="n">
+        <v>296.6</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>185.741586303711</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>110.8584136962891</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0.6262359619140625</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>0.1061877309819517</v>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>ZEBRE</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>{'total_capex': 296.6, 'debt_amount': 192.78926456451418, 'equity_amount': 103.81073543548585, 'gearing': 0.6499975204467774}</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
         <is>
           <t>QLD</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr">
+      <c r="AQ6" t="inlineStr">
         <is>
           <t>2028-05-01</t>
-        </is>
-      </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>2.00</t>
-        </is>
-      </c>
-      <c r="Y6" t="n">
-        <v>5.19</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>83</v>
-      </c>
-      <c r="AB6" t="n">
-        <v>296.6</v>
-      </c>
-      <c r="AC6" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="AD6" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="AE6" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="AF6" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="AG6" t="n">
-        <v>20</v>
-      </c>
-      <c r="AH6" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="AI6" t="inlineStr">
-        <is>
-          <t>sculpting</t>
-        </is>
-      </c>
-      <c r="AJ6" t="n">
-        <v>296.6</v>
-      </c>
-      <c r="AK6" t="n">
-        <v>192.7892645645142</v>
-      </c>
-      <c r="AL6" t="n">
-        <v>103.8107354354859</v>
-      </c>
-      <c r="AM6" t="n">
-        <v>0.6499975204467774</v>
-      </c>
-      <c r="AN6" t="n">
-        <v>0.1607519897242499</v>
-      </c>
-      <c r="AO6" t="inlineStr">
-        <is>
-          <t>ZEBRE</t>
-        </is>
-      </c>
-      <c r="AP6" t="inlineStr"/>
-      <c r="AQ6" t="inlineStr">
-        <is>
-          <t>{'total_capex': 296.6, 'debt_amount': 192.78926456451418, 'equity_amount': 103.81073543548585, 'gearing': 0.6499975204467774}</t>
         </is>
       </c>
     </row>
@@ -1468,92 +1446,92 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
+          <t>4.00</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
           <t>[{'id': '1', 'counterparty': 'ZEN', 'type': 'tolling', 'buyersPercentage': 100, 'shape': 'flat', 'strikePrice': 20, 'greenPrice': '', 'EnergyPrice': '', 'indexation': 2.5, 'indexationReferenceYear': '2025', 'settlementFormula': '', 'hasFloor': False, 'floorValue': '', 'startDate': '2028-05-01', 'endDate': '2038-04-30'}]</t>
         </is>
       </c>
-      <c r="S7" t="n">
+      <c r="T7" t="n">
         <v>6</v>
       </c>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr">
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr">
         <is>
           <t>{'operatingCosts': 5.95, 'operatingCostEscalation': 2.5, 'terminalValue': 93, 'capex': 452.7, 'maxGearing': 0.65, 'targetDSCRContract': 1.4, 'targetDSCRMerchant': 1.8, 'interestRate': 0.06, 'tenorYears': 20, 'calculatedGearing': 0.65, 'debtStructure': 'sculpting'}</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="W7" t="n">
+        <v>5.95</v>
+      </c>
+      <c r="X7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>93</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>452.7</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>20</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>sculpting</t>
+        </is>
+      </c>
+      <c r="AH7" t="n">
+        <v>452.7</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>232.9674028301239</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>219.7325971698761</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>0.51461763381958</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>0.09215721287554127</v>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>ZEBRE</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr"/>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>{'total_capex': 452.70000000000005, 'debt_amount': 294.25443875312806, 'equity_amount': 158.44556124687196, 'gearing': 0.6499987602233886}</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
         <is>
           <t>NSW</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr">
+      <c r="AQ7" t="inlineStr">
         <is>
           <t>2028-05-01</t>
-        </is>
-      </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>4.00</t>
-        </is>
-      </c>
-      <c r="Y7" t="n">
-        <v>5.95</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>93</v>
-      </c>
-      <c r="AB7" t="n">
-        <v>452.7</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="AE7" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="AF7" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="AG7" t="n">
-        <v>20</v>
-      </c>
-      <c r="AH7" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="AI7" t="inlineStr">
-        <is>
-          <t>sculpting</t>
-        </is>
-      </c>
-      <c r="AJ7" t="n">
-        <v>452.7</v>
-      </c>
-      <c r="AK7" t="n">
-        <v>294.2544387531281</v>
-      </c>
-      <c r="AL7" t="n">
-        <v>158.445561246872</v>
-      </c>
-      <c r="AM7" t="n">
-        <v>0.6499987602233886</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>0.136922849696032</v>
-      </c>
-      <c r="AO7" t="inlineStr">
-        <is>
-          <t>ZEBRE</t>
-        </is>
-      </c>
-      <c r="AP7" t="inlineStr"/>
-      <c r="AQ7" t="inlineStr">
-        <is>
-          <t>{'total_capex': 452.70000000000005, 'debt_amount': 294.25443875312806, 'equity_amount': 158.44556124687196, 'gearing': 0.6499987602233886}</t>
         </is>
       </c>
     </row>
@@ -1617,92 +1595,92 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
+          <t>4.00</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
           <t>[{'id': '1', 'counterparty': 'ZEN Tolling', 'type': 'tolling', 'buyersPercentage': 100, 'shape': 'flat', 'strikePrice': 20, 'greenPrice': '', 'EnergyPrice': '', 'indexation': 2.5, 'indexationReferenceYear': '2025', 'settlementFormula': '', 'hasFloor': False, 'floorValue': '', 'startDate': '2029-05-01', 'endDate': '2039-04-30'}]</t>
         </is>
       </c>
-      <c r="S8" t="n">
+      <c r="T8" t="n">
         <v>7</v>
       </c>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr">
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr">
         <is>
           <t>{'operatingCosts': 6.05, 'operatingCostEscalation': 2.5, 'terminalValue': 97, 'capex': 512.7, 'maxGearing': 0.65, 'targetDSCRContract': 1.4, 'targetDSCRMerchant': 1.8, 'interestRate': 0.06, 'tenorYears': 20, 'calculatedGearing': 0.65, 'debtStructure': 'sculpting'}</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="W8" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="X8" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>97</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>512.7</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>20</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>sculpting</t>
+        </is>
+      </c>
+      <c r="AH8" t="n">
+        <v>512.7000000000002</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>246.1941907024383</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>266.5058092975618</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>0.4801915168762205</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>0.08966351230365671</v>
+      </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>ZEBRE</t>
+        </is>
+      </c>
+      <c r="AN8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>{'total_capex': 512.7000000000002, 'debt_amount': 333.2543643665313, 'equity_amount': 179.44563563346878, 'gearing': 0.6499987602233883}</t>
+        </is>
+      </c>
+      <c r="AP8" t="inlineStr">
         <is>
           <t>VIC</t>
         </is>
       </c>
-      <c r="W8" t="inlineStr">
+      <c r="AQ8" t="inlineStr">
         <is>
           <t>2029-05-01</t>
-        </is>
-      </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>4.00</t>
-        </is>
-      </c>
-      <c r="Y8" t="n">
-        <v>6.05</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="AA8" t="n">
-        <v>97</v>
-      </c>
-      <c r="AB8" t="n">
-        <v>512.7</v>
-      </c>
-      <c r="AC8" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="AD8" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="AE8" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="AF8" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="AG8" t="n">
-        <v>20</v>
-      </c>
-      <c r="AH8" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="AI8" t="inlineStr">
-        <is>
-          <t>sculpting</t>
-        </is>
-      </c>
-      <c r="AJ8" t="n">
-        <v>512.7000000000002</v>
-      </c>
-      <c r="AK8" t="n">
-        <v>333.2543643665313</v>
-      </c>
-      <c r="AL8" t="n">
-        <v>179.4456356334688</v>
-      </c>
-      <c r="AM8" t="n">
-        <v>0.6499987602233883</v>
-      </c>
-      <c r="AN8" t="n">
-        <v>0.1324552854535143</v>
-      </c>
-      <c r="AO8" t="inlineStr">
-        <is>
-          <t>ZEBRE</t>
-        </is>
-      </c>
-      <c r="AP8" t="inlineStr"/>
-      <c r="AQ8" t="inlineStr">
-        <is>
-          <t>{'total_capex': 512.7000000000002, 'debt_amount': 333.2543643665313, 'equity_amount': 179.44563563346878, 'gearing': 0.6499987602233883}</t>
         </is>
       </c>
     </row>
@@ -1764,92 +1742,92 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
           <t>[{'id': '1', 'counterparty': 'ZEN Tolling', 'type': 'tolling', 'buyersPercentage': 100, 'shape': 'flat', 'strikePrice': 21, 'greenPrice': '', 'EnergyPrice': '', 'indexation': '2.5', 'indexationReferenceYear': '2025', 'settlementFormula': '', 'hasFloor': False, 'floorValue': '', 'startDate': '2028-01-01', 'endDate': '2037-12-31'}]</t>
         </is>
       </c>
-      <c r="S9" t="n">
+      <c r="T9" t="n">
         <v>8</v>
       </c>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr">
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr">
         <is>
           <t>{'capex': 141.5, 'operatingCosts': 2.2, 'operatingCostEscalation': 2.5, 'terminalValue': 32, 'maxGearing': 0.7, 'targetDSCRContract': 1.4, 'targetDSCRMerchant': 2, 'interestRate': 0.06, 'tenorYears': 18, 'debtStructure': 'sculpting', 'calculatedGearing': 0.7}</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
+      <c r="W9" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="X9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>32</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>141.5</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>18</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>sculpting</t>
+        </is>
+      </c>
+      <c r="AH9" t="n">
+        <v>141.5</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>95.60480232238771</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>45.89519767761228</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0.675652313232422</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>0.1246654272106846</v>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>ZEBRE</t>
+        </is>
+      </c>
+      <c r="AN9" t="inlineStr"/>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>{'total_capex': 141.5, 'debt_amount': 94.51887359619141, 'equity_amount': 46.98112640380858, 'gearing': 0.6679779052734376}</t>
+        </is>
+      </c>
+      <c r="AP9" t="inlineStr">
         <is>
           <t>VIC</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr">
+      <c r="AQ9" t="inlineStr">
         <is>
           <t>2028-01-01</t>
-        </is>
-      </c>
-      <c r="X9" t="inlineStr">
-        <is>
-          <t>3.00</t>
-        </is>
-      </c>
-      <c r="Y9" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="AA9" t="n">
-        <v>32</v>
-      </c>
-      <c r="AB9" t="n">
-        <v>141.5</v>
-      </c>
-      <c r="AC9" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AD9" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="AE9" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF9" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="AG9" t="n">
-        <v>18</v>
-      </c>
-      <c r="AH9" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AI9" t="inlineStr">
-        <is>
-          <t>sculpting</t>
-        </is>
-      </c>
-      <c r="AJ9" t="n">
-        <v>141.5</v>
-      </c>
-      <c r="AK9" t="n">
-        <v>95.60102386474611</v>
-      </c>
-      <c r="AL9" t="n">
-        <v>45.89897613525388</v>
-      </c>
-      <c r="AM9" t="n">
-        <v>0.6756256103515627</v>
-      </c>
-      <c r="AN9" t="n">
-        <v>0.1721991906314946</v>
-      </c>
-      <c r="AO9" t="inlineStr">
-        <is>
-          <t>ZEBRE</t>
-        </is>
-      </c>
-      <c r="AP9" t="inlineStr"/>
-      <c r="AQ9" t="inlineStr">
-        <is>
-          <t>{'total_capex': 141.5, 'debt_amount': 94.51887359619141, 'equity_amount': 46.98112640380858, 'gearing': 0.6679779052734376}</t>
         </is>
       </c>
     </row>
@@ -2100,13 +2078,13 @@
         <v>500</v>
       </c>
       <c r="C4" t="n">
-        <v>337.9670143127441</v>
+        <v>297.6076126098633</v>
       </c>
       <c r="D4" t="n">
-        <v>162.0329856872559</v>
+        <v>202.3923873901367</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6759340286254882</v>
+        <v>0.5952152252197267</v>
       </c>
     </row>
     <row r="5">
@@ -2119,13 +2097,13 @@
         <v>246.8</v>
       </c>
       <c r="C5" t="n">
-        <v>160.4193880462647</v>
+        <v>121.4581295776367</v>
       </c>
       <c r="D5" t="n">
-        <v>86.38061195373534</v>
+        <v>125.3418704223633</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6499975204467774</v>
+        <v>0.4921318054199219</v>
       </c>
     </row>
     <row r="6">
@@ -2138,13 +2116,13 @@
         <v>296.6</v>
       </c>
       <c r="C6" t="n">
-        <v>192.7892645645142</v>
+        <v>185.741586303711</v>
       </c>
       <c r="D6" t="n">
-        <v>103.8107354354859</v>
+        <v>110.8584136962891</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6499975204467774</v>
+        <v>0.6262359619140625</v>
       </c>
     </row>
     <row r="7">
@@ -2157,13 +2135,13 @@
         <v>452.7</v>
       </c>
       <c r="C7" t="n">
-        <v>294.2544387531281</v>
+        <v>232.9674028301239</v>
       </c>
       <c r="D7" t="n">
-        <v>158.445561246872</v>
+        <v>219.7325971698761</v>
       </c>
       <c r="E7" t="n">
-        <v>0.6499987602233886</v>
+        <v>0.51461763381958</v>
       </c>
     </row>
     <row r="8">
@@ -2176,13 +2154,13 @@
         <v>512.7000000000002</v>
       </c>
       <c r="C8" t="n">
-        <v>333.2543643665313</v>
+        <v>246.1941907024383</v>
       </c>
       <c r="D8" t="n">
-        <v>179.4456356334688</v>
+        <v>266.5058092975618</v>
       </c>
       <c r="E8" t="n">
-        <v>0.6499987602233883</v>
+        <v>0.4801915168762205</v>
       </c>
     </row>
     <row r="9">
@@ -2195,13 +2173,13 @@
         <v>141.5</v>
       </c>
       <c r="C9" t="n">
-        <v>95.60102386474611</v>
+        <v>95.60480232238771</v>
       </c>
       <c r="D9" t="n">
-        <v>45.89897613525388</v>
+        <v>45.89519767761228</v>
       </c>
       <c r="E9" t="n">
-        <v>0.6756256103515627</v>
+        <v>0.675652313232422</v>
       </c>
     </row>
   </sheetData>
@@ -2227,7 +2205,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.158395181268125</v>
+        <v>0.1022691457886931</v>
       </c>
     </row>
   </sheetData>
@@ -2261,7 +2239,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>0.1436087041880745</v>
+        <v>0.09946314289147172</v>
       </c>
     </row>
     <row r="3">
@@ -2269,7 +2247,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>0.2838806754680757</v>
+        <v>0.2104294561684678</v>
       </c>
     </row>
     <row r="4">
@@ -2277,7 +2255,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>0.1623527630417089</v>
+        <v>0.07631405246890151</v>
       </c>
     </row>
     <row r="5">
@@ -2285,7 +2263,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>0.1305817350477535</v>
+        <v>0.08692668341712489</v>
       </c>
     </row>
     <row r="6">
@@ -2293,7 +2271,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>0.1607519897242499</v>
+        <v>0.1061877309819517</v>
       </c>
     </row>
     <row r="7">
@@ -2301,7 +2279,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>0.136922849696032</v>
+        <v>0.09215721287554127</v>
       </c>
     </row>
     <row r="8">
@@ -2309,7 +2287,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>0.1324552854535143</v>
+        <v>0.08966351230365671</v>
       </c>
     </row>
     <row r="9">
@@ -2317,7 +2295,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>0.1721991906314946</v>
+        <v>0.1246654272106846</v>
       </c>
     </row>
   </sheetData>

</xml_diff>